<commit_message>
fiddling with things for caras check in
</commit_message>
<xml_diff>
--- a/EstsAndpValues02.xlsx
+++ b/EstsAndpValues02.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/474cc55cc2f2a489/Desktop/Fall2025PoolsAnalysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_AA2BA2750CD1698BCB624D77B8AAEC2FFAC83429" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{062F2D68-D8A7-4EB3-9768-32AF03BDAE34}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_AA2BA2750CD1698BCB624D77B8AAEC2FFAC83429" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32DD55FF-953A-4409-BAAE-8D0FE6FA35A6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ests_Overall" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -82,12 +82,101 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -388,322 +477,322 @@
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
+      <c r="A2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5">
         <v>0.25876074142140698</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="5">
         <v>0.22771105544505699</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="5">
         <v>0.24569412846758201</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="5">
         <v>0.323621420793481</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="5">
         <v>0.24217536466199499</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="5">
         <v>0.51637855583693104</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="5">
         <v>0.27888802205500302</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="6">
         <v>0.283254066135805</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="5">
         <v>0.25876074142140698</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
+      <c r="C3" s="5">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5">
         <v>0.71428167630804695</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="5">
         <v>0.68856711234590895</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="5">
         <v>0.69819296695497601</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="5">
         <v>0.60428224053410395</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="5">
         <v>0.31984222762039</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="5">
         <v>0.57542355871106099</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="6">
         <v>0.60293548259899998</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="5">
         <v>0.22771105544505699</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="5">
         <v>0.71428167630804695</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
+      <c r="D4" s="5">
+        <v>1</v>
+      </c>
+      <c r="E4" s="5">
         <v>0.71260818055904296</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="5">
         <v>0.71457228614838098</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="5">
         <v>0.69191186249123904</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="5">
         <v>0.261602273210439</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="5">
         <v>0.56164436484576497</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="6">
         <v>0.49790895752394698</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="5">
         <v>0.24569412846758201</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="5">
         <v>0.68856711234590895</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="5">
         <v>0.71260818055904296</v>
       </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
+      <c r="E5" s="5">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5">
         <v>0.62063721924603898</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="5">
         <v>0.62582663081754597</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="5">
         <v>0.25115032181182301</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="5">
         <v>0.60665203251413902</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="6">
         <v>0.52046878271502095</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="5">
         <v>0.323621420793481</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="5">
         <v>0.69819296695497601</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="5">
         <v>0.71457228614838098</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="5">
         <v>0.62063721924603898</v>
       </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
+      <c r="F6" s="5">
+        <v>1</v>
+      </c>
+      <c r="G6" s="5">
         <v>0.64499909238631103</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="5">
         <v>0.35404133151211298</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="5">
         <v>0.62269521393749405</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="6">
         <v>0.53808643823983804</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="5">
         <v>0.24217536466199499</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="5">
         <v>0.60428224053410395</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="5">
         <v>0.69191186249123904</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="5">
         <v>0.62582663081754597</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="5">
         <v>0.64499909238631103</v>
       </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="H7">
+      <c r="G7" s="5">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5">
         <v>0.25576615383039603</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="5">
         <v>0.46188312480869198</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="6">
         <v>0.43521955056006101</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="5">
         <v>0.51637855583693104</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="5">
         <v>0.31984222762039</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="5">
         <v>0.261602273210439</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="5">
         <v>0.25115032181182301</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="5">
         <v>0.35404133151211298</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="5">
         <v>0.25576615383039603</v>
       </c>
-      <c r="H8">
-        <v>1</v>
-      </c>
-      <c r="I8">
+      <c r="H8" s="5">
+        <v>1</v>
+      </c>
+      <c r="I8" s="5">
         <v>0.328501641328937</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="6">
         <v>0.36565531563723702</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="5">
         <v>0.27888802205500302</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="5">
         <v>0.57542355871106099</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="5">
         <v>0.56164436484576497</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="5">
         <v>0.60665203251413902</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="5">
         <v>0.62269521393749405</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="5">
         <v>0.46188312480869198</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="5">
         <v>0.328501641328937</v>
       </c>
-      <c r="I9">
-        <v>1</v>
-      </c>
-      <c r="J9">
+      <c r="I9" s="5">
+        <v>1</v>
+      </c>
+      <c r="J9" s="6">
         <v>0.53916132412218698</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="10" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="8">
         <v>0.283254066135805</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="8">
         <v>0.60293548259899998</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="8">
         <v>0.49790895752394698</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="8">
         <v>0.52046878271502095</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="8">
         <v>0.53808643823983804</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="8">
         <v>0.43521955056006101</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="8">
         <v>0.36565531563723702</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="8">
         <v>0.53916132412218698</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="9">
         <v>1</v>
       </c>
     </row>

</xml_diff>